<commit_message>
feat: Them cot Dan Toc vao GSheet va DB - database.py: them cot dan_toc vao migration - app.py: them API /api/student-ethnicity (tra CCCD->dan_toc) - app.py: import Excel doc truong dan_toc - tsdc_push.py: fetch dan_toc tu DB, map qua CCCD - Code.gs: them cot Dan toc (col 15) truoc Cap nhat luc - Template: them cot dan_toc vao file mau
</commit_message>
<xml_diff>
--- a/data/students_template.xlsx
+++ b/data/students_template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,6 +444,11 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>dan_toc</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>ghi_chu</t>
         </is>
       </c>
@@ -474,7 +479,6 @@
           <t>12/05/2011</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -502,7 +506,6 @@
           <t>21/08/2011</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -530,7 +533,6 @@
           <t>05/03/2011</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -558,7 +560,6 @@
           <t>17/01/2011</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -586,7 +587,6 @@
           <t>09/11/2011</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -614,7 +614,6 @@
           <t>28/06/2011</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>